<commit_message>
updates on 20 mar
</commit_message>
<xml_diff>
--- a/LangGraph/eval_skeleton (LangGraph).xlsx
+++ b/LangGraph/eval_skeleton (LangGraph).xlsx
@@ -9721,31 +9721,31 @@
         <v>0</v>
       </c>
       <c r="J209" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K209" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="K209" s="18" t="n">
-        <v>0.8</v>
-      </c>
       <c r="L209" s="18" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="M209" s="18" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="N209" s="18" t="n">
-        <v>0.3043478260869565</v>
+        <v>0.5925925925925926</v>
       </c>
       <c r="O209" s="18" t="n">
-        <v>0.2258064516129032</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="P209" s="18" t="n">
-        <v>0.4666666666666667</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="Q209" s="18" t="n">
         <v>1</v>
       </c>
       <c r="R209" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210" ht="15.75" customHeight="1" s="66">
@@ -9919,7 +9919,7 @@
         <v>0</v>
       </c>
       <c r="J213" s="18" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K213" s="18" t="n">
         <v>1</v>
@@ -9931,13 +9931,13 @@
         <v>0</v>
       </c>
       <c r="N213" s="18" t="n">
-        <v>0</v>
+        <v>0.2040816326530612</v>
       </c>
       <c r="O213" s="18" t="n">
-        <v>0</v>
+        <v>0.1219512195121951</v>
       </c>
       <c r="P213" s="18" t="n">
-        <v>0</v>
+        <v>0.625</v>
       </c>
       <c r="Q213" s="18" t="n">
         <v>0</v>
@@ -10243,34 +10243,34 @@
         </is>
       </c>
       <c r="H219" s="18" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="I219" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J219" s="18" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K219" s="18" t="n">
         <v>1</v>
-      </c>
-      <c r="J219" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K219" s="18" t="n">
-        <v>0</v>
       </c>
       <c r="L219" s="18" t="n">
         <v>0</v>
       </c>
       <c r="M219" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N219" s="18" t="n">
-        <v>0.4782608695652174</v>
+        <v>0.3050847457627118</v>
       </c>
       <c r="O219" s="18" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.2093023255813954</v>
       </c>
       <c r="P219" s="18" t="n">
-        <v>0.34375</v>
+        <v>0.5625</v>
       </c>
       <c r="Q219" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R219" s="18" t="n">
         <v>0</v>
@@ -10359,28 +10359,28 @@
         <v>0</v>
       </c>
       <c r="J221" s="18" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="K221" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L221" s="18" t="n">
         <v>0</v>
       </c>
       <c r="M221" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N221" s="18" t="n">
-        <v>0.08823529411764705</v>
+        <v>0.1866666666666666</v>
       </c>
       <c r="O221" s="18" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.1076923076923077</v>
       </c>
       <c r="P221" s="18" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="Q221" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R221" s="18" t="n">
         <v>0</v>
@@ -10667,7 +10667,7 @@
         <v>0</v>
       </c>
       <c r="J227" s="18" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K227" s="18" t="n">
         <v>1</v>
@@ -10679,13 +10679,13 @@
         <v>0</v>
       </c>
       <c r="N227" s="18" t="n">
-        <v>0.36</v>
+        <v>0.0396694214876033</v>
       </c>
       <c r="O227" s="18" t="n">
-        <v>0.2368421052631579</v>
+        <v>0.02023608768971332</v>
       </c>
       <c r="P227" s="18" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="Q227" s="18" t="n">
         <v>1</v>
@@ -11085,31 +11085,31 @@
         <v>0</v>
       </c>
       <c r="J236" s="18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K236" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L236" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M236" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="K236" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L236" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M236" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="N236" s="18" t="n">
-        <v>0.2</v>
+        <v>0.0704225352112676</v>
       </c>
       <c r="O236" s="18" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.03712871287128713</v>
       </c>
       <c r="P236" s="18" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="Q236" s="18" t="n">
         <v>1</v>
       </c>
       <c r="R236" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237" ht="15.75" customHeight="1" s="66">
@@ -11371,28 +11371,28 @@
         <v>0</v>
       </c>
       <c r="J242" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K242" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L242" s="18" t="n">
         <v>0</v>
       </c>
       <c r="M242" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N242" s="18" t="n">
-        <v>0.2033898305084746</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="O242" s="18" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1228070175438596</v>
       </c>
       <c r="P242" s="18" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="Q242" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R242" s="18" t="n">
         <v>0</v>
@@ -11481,31 +11481,31 @@
         <v>1</v>
       </c>
       <c r="J244" s="18" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K244" s="18" t="n">
         <v>1</v>
       </c>
       <c r="L244" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M244" s="18" t="n">
         <v>0</v>
       </c>
       <c r="N244" s="18" t="n">
-        <v>0.2444444444444444</v>
+        <v>0.1185983827493261</v>
       </c>
       <c r="O244" s="18" t="n">
-        <v>0.1896551724137931</v>
+        <v>0.06489675516224189</v>
       </c>
       <c r="P244" s="18" t="n">
-        <v>0.34375</v>
+        <v>0.6875</v>
       </c>
       <c r="Q244" s="18" t="n">
         <v>1</v>
       </c>
       <c r="R244" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="245" ht="15.75" customHeight="1" s="66">
@@ -11547,25 +11547,25 @@
         <v>0</v>
       </c>
       <c r="J245" s="18" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K245" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L245" s="18" t="n">
         <v>0</v>
       </c>
       <c r="M245" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N245" s="18" t="n">
-        <v>0.1935483870967742</v>
+        <v>0.05882352941176471</v>
       </c>
       <c r="O245" s="18" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.03038674033149171</v>
       </c>
       <c r="P245" s="18" t="n">
-        <v>0.25</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="Q245" s="18" t="n">
         <v>1</v>
@@ -13540,9 +13540,7 @@
       <c r="M285" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="N285" s="18" t="n">
-        <v/>
-      </c>
+      <c r="N285" s="18" t="n"/>
       <c r="O285" s="18" t="n">
         <v>0</v>
       </c>
@@ -13600,9 +13598,7 @@
       <c r="M286" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="N286" s="18" t="n">
-        <v/>
-      </c>
+      <c r="N286" s="18" t="n"/>
       <c r="O286" s="18" t="n">
         <v>0</v>
       </c>
@@ -13698,9 +13694,7 @@
       <c r="M288" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="N288" s="18" t="n">
-        <v/>
-      </c>
+      <c r="N288" s="18" t="n"/>
       <c r="O288" s="18" t="n">
         <v>0</v>
       </c>
@@ -13834,9 +13828,7 @@
       <c r="M291" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="N291" s="18" t="n">
-        <v/>
-      </c>
+      <c r="N291" s="18" t="n"/>
       <c r="O291" s="18" t="n">
         <v>0</v>
       </c>
@@ -13894,9 +13886,7 @@
       <c r="M292" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="N292" s="18" t="n">
-        <v/>
-      </c>
+      <c r="N292" s="18" t="n"/>
       <c r="O292" s="18" t="n">
         <v>0</v>
       </c>
@@ -14128,9 +14118,7 @@
       <c r="M297" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="N297" s="18" t="n">
-        <v/>
-      </c>
+      <c r="N297" s="18" t="n"/>
       <c r="O297" s="18" t="n">
         <v>0</v>
       </c>

</xml_diff>